<commit_message>
chore: run 2026-03-13 22:39 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_13_03_2026.xlsx
+++ b/logs/Consolidado_13_03_2026.xlsx
@@ -657,10 +657,10 @@
         <v>65</v>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>
@@ -9123,40 +9123,40 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>13/03/2026</t>
-        </is>
-      </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>13/03/2026</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr">
+      <c r="C47" s="7" t="inlineStr">
         <is>
           <t>Keracnyl Repair Baume Lèvres
 Bálsamo Lábios Gretados e Danificados Acne
 15 ml</t>
         </is>
       </c>
-      <c r="D47" s="3" t="inlineStr">
+      <c r="D47" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/keracnyl-repair-baume-levres-5410512.html</t>
         </is>
       </c>
-      <c r="E47" s="3" t="inlineStr"/>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G47" s="3" t="inlineStr">
+      <c r="E47" s="7" t="inlineStr"/>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G47" s="7" t="inlineStr">
         <is>
           <t>5410512</t>
         </is>
       </c>
-      <c r="H47" s="3" t="inlineStr">
+      <c r="H47" s="7" t="inlineStr">
         <is>
           <t>25%</t>
         </is>

</xml_diff>